<commit_message>
Biologiplanering: syfte, centralt innehåll och förmåga som text i stället för koder
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017mqJrSEX6tzqa8YfkctM6P
</commit_message>
<xml_diff>
--- a/planering/biologi-planering.xlsx
+++ b/planering/biologi-planering.xlsx
@@ -496,7 +496,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Syftesdelar härleds: F1→S2, F3→S7, SU3→S6, SU4→S4. S1, S3, S5, S8 är satta för hand.</t>
+          <t>Syfte: den del av ämnets syfte (i sak) som momentet bygger på. Delar som följer av förmåga eller innehåll är härledda automatiskt.</t>
         </is>
       </c>
     </row>
@@ -659,17 +659,17 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>S1 Nyfikenhet och frågor; S7 Systematiska undersökningar</t>
+          <t>Nyfikenhet och intresse; ställa frågor om natur och människa utifrån egna upplevelser och aktuella händelser; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -722,17 +722,17 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -785,17 +785,17 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -848,17 +848,17 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar; S8 Material, utrustning, digitalt</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder; Färdigheter i att hantera material, utrustning och digitala verktyg</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -907,13 +907,13 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>S1 Nyfikenhet och frågor; S2 Begrepp och samband</t>
+          <t>Nyfikenhet och intresse; ställa frågor om natur och människa utifrån egna upplevelser och aktuella händelser; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -962,17 +962,17 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>S1 Nyfikenhet och frågor; S7 Systematiska undersökningar</t>
+          <t>Nyfikenhet och intresse; ställa frågor om natur och människa utifrån egna upplevelser och aktuella händelser; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -1021,17 +1021,17 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -1084,17 +1084,17 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S6 Källor och kritiskt tänkande</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>SU3 Informationsgranskning</t>
+          <t>Informationsgranskning</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -1147,17 +1147,17 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar; S2 Begrepp och samband</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>SU2 Modeller och historia</t>
+          <t>Modeller och historia</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -1210,17 +1210,17 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>SU3 Informationsgranskning</t>
+          <t>Informationsgranskning</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -1273,17 +1273,17 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>SU3 Informationsgranskning</t>
+          <t>Informationsgranskning</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -1332,17 +1332,17 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>SU2 Modeller och historia</t>
+          <t>Modeller och historia</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>SU2 Modeller och historia</t>
+          <t>Modeller och historia</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr"/>
@@ -1446,17 +1446,17 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>SU3 Informationsgranskning</t>
+          <t>Informationsgranskning</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -1505,17 +1505,17 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>SU3 Informationsgranskning; SU1 Undersökningar</t>
+          <t>Informationsgranskning; Undersökningar</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -1564,17 +1564,17 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>S4 Argument och kommunikation</t>
+          <t>Formulera egna och granska andras argument; kommunicera</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>SU4 Argumentation</t>
+          <t>Argumentation</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -1627,17 +1627,17 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; SU2 Modeller och historia</t>
+          <t>Celler och organsystem; Modeller och historia</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -1690,17 +1690,17 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -1753,17 +1753,17 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -1816,17 +1816,17 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; SU1 Undersökningar</t>
+          <t>Celler och organsystem; Undersökningar</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -1875,17 +1875,17 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband; S7 Systematiska undersökningar</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller; F3 Undersöka</t>
+          <t>Begrepp/modeller; Undersöka</t>
         </is>
       </c>
     </row>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr"/>
@@ -1993,17 +1993,17 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2056,17 +2056,17 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; KH1 Celler och organsystem</t>
+          <t>Fotosyntes, kretslopp, energi; Celler och organsystem</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2119,17 +2119,17 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2182,17 +2182,17 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; SU1 Undersökningar</t>
+          <t>Fotosyntes, kretslopp, energi; Undersökningar</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -2241,17 +2241,17 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; KH1 Celler och organsystem</t>
+          <t>Fotosyntes, kretslopp, energi; Celler och organsystem</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2300,17 +2300,17 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; SU1 Undersökningar</t>
+          <t>Fotosyntes, kretslopp, energi; Undersökningar</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -2359,17 +2359,17 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2418,17 +2418,17 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2481,17 +2481,17 @@
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2544,17 +2544,17 @@
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2603,17 +2603,17 @@
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2666,17 +2666,17 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM6 Påverkan och hållbarhet</t>
+          <t>Evolution och mångfald; Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2729,17 +2729,17 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2792,17 +2792,17 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -2855,17 +2855,17 @@
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet; SU1 Undersökningar</t>
+          <t>Påverkan och hållbarhet; Undersökningar</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -2914,17 +2914,17 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet; SU1 Undersökningar</t>
+          <t>Påverkan och hållbarhet; Undersökningar</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -2973,17 +2973,17 @@
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM4 Ekosystem och populationer</t>
+          <t>Evolution och mångfald; Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3036,17 +3036,17 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3099,17 +3099,17 @@
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3162,17 @@
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3225,17 +3225,17 @@
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; SU1 Undersökningar</t>
+          <t>Evolution och mångfald; Undersökningar</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -3284,17 +3284,17 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3343,17 +3343,17 @@
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3402,17 +3402,17 @@
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3461,17 +3461,17 @@
       </c>
       <c r="K48" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3520,17 +3520,17 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM4 Ekosystem och populationer</t>
+          <t>Evolution och mångfald; Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3579,17 +3579,17 @@
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3638,17 +3638,17 @@
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3701,17 +3701,17 @@
       </c>
       <c r="K52" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer</t>
+          <t>Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3764,17 +3764,17 @@
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer; NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Ekosystem och populationer; Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,17 @@
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -3890,17 +3890,17 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; SU1 Undersökningar</t>
+          <t>Fotosyntes, kretslopp, energi; Undersökningar</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -3949,17 +3949,17 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer</t>
+          <t>Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4008,17 +4008,17 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer</t>
+          <t>Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4067,17 +4067,17 @@
       </c>
       <c r="K58" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer; NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Ekosystem och populationer; Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4127,12 +4127,12 @@
       <c r="K59" s="4" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer</t>
+          <t>Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -4185,17 +4185,17 @@
       </c>
       <c r="K60" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4248,17 +4248,17 @@
       </c>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4311,17 +4311,17 @@
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4374,17 +4374,17 @@
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; SU1 Undersökningar</t>
+          <t>Fotosyntes, kretslopp, energi; Undersökningar</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -4433,17 +4433,17 @@
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4496,17 +4496,17 @@
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer; SU1 Undersökningar</t>
+          <t>Ekosystem och populationer; Undersökningar</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4559,17 +4559,17 @@
       </c>
       <c r="K66" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer</t>
+          <t>Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4622,17 +4622,17 @@
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer; NM1 Evolution och mångfald</t>
+          <t>Ekosystem och populationer; Evolution och mångfald</t>
         </is>
       </c>
       <c r="M67" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4685,17 +4685,17 @@
       </c>
       <c r="K68" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer; SU1 Undersökningar</t>
+          <t>Ekosystem och populationer; Undersökningar</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -4744,17 +4744,17 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>NM4 Ekosystem och populationer</t>
+          <t>Ekosystem och populationer</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4807,17 +4807,17 @@
       </c>
       <c r="K70" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M70" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4870,17 +4870,17 @@
       </c>
       <c r="K71" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L71" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; NM6 Påverkan och hållbarhet</t>
+          <t>Fotosyntes, kretslopp, energi; Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M71" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4933,17 +4933,17 @@
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L72" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M72" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -4996,17 +4996,17 @@
       </c>
       <c r="K73" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; NM6 Påverkan och hållbarhet; SU1 Undersökningar</t>
+          <t>Fotosyntes, kretslopp, energi; Påverkan och hållbarhet; Undersökningar</t>
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -5055,17 +5055,17 @@
       </c>
       <c r="K74" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L74" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M74" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5114,17 +5114,17 @@
       </c>
       <c r="K75" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L75" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet; NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Påverkan och hållbarhet; Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M75" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5173,17 +5173,17 @@
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L76" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M76" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5233,12 +5233,12 @@
       <c r="K77" s="4" t="inlineStr"/>
       <c r="L77" s="4" t="inlineStr">
         <is>
-          <t>NM5 Fotosyntes, kretslopp, energi; NM6 Påverkan och hållbarhet</t>
+          <t>Fotosyntes, kretslopp, energi; Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M77" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -5291,17 +5291,17 @@
       </c>
       <c r="K78" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val; S2 Begrepp och samband</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L78" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M78" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5354,17 +5354,17 @@
       </c>
       <c r="K79" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L79" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M79" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5417,17 +5417,17 @@
       </c>
       <c r="K80" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L80" s="4" t="inlineStr">
         <is>
-          <t>NM6 Påverkan och hållbarhet</t>
+          <t>Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M80" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -5480,17 +5480,17 @@
       </c>
       <c r="K81" s="4" t="inlineStr">
         <is>
-          <t>S4 Argument och kommunikation; S5 Etiska val</t>
+          <t>Formulera egna och granska andras argument; kommunicera; Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L81" s="4" t="inlineStr">
         <is>
-          <t>SU4 Argumentation</t>
+          <t>Argumentation</t>
         </is>
       </c>
       <c r="M81" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -5539,17 +5539,17 @@
       </c>
       <c r="K82" s="4" t="inlineStr">
         <is>
-          <t>S4 Argument och kommunikation; S5 Etiska val</t>
+          <t>Formulera egna och granska andras argument; kommunicera; Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L82" s="4" t="inlineStr">
         <is>
-          <t>SU4 Argumentation</t>
+          <t>Argumentation</t>
         </is>
       </c>
       <c r="M82" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -5602,17 +5602,17 @@
       </c>
       <c r="K83" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L83" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; KH3 Hälsa</t>
+          <t>Celler och organsystem; Hälsa</t>
         </is>
       </c>
       <c r="M83" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5665,17 +5665,17 @@
       </c>
       <c r="K84" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L84" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M84" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5728,17 +5728,17 @@
       </c>
       <c r="K85" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L85" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M85" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5791,17 +5791,17 @@
       </c>
       <c r="K86" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L86" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; SU1 Undersökningar</t>
+          <t>Celler och organsystem; Undersökningar</t>
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -5850,17 +5850,17 @@
       </c>
       <c r="K87" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L87" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; KH3 Hälsa</t>
+          <t>Celler och organsystem; Hälsa</t>
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5909,17 +5909,17 @@
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M88" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -5968,17 +5968,17 @@
       </c>
       <c r="K89" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L89" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M89" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6027,17 +6027,17 @@
       </c>
       <c r="K90" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L90" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; KH2 Infektioner</t>
+          <t>Celler och organsystem; Infektioner</t>
         </is>
       </c>
       <c r="M90" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6087,12 +6087,12 @@
       <c r="K91" s="4" t="inlineStr"/>
       <c r="L91" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; NM6 Påverkan och hållbarhet</t>
+          <t>Hälsa; Påverkan och hållbarhet</t>
         </is>
       </c>
       <c r="M91" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -6141,17 +6141,17 @@
       </c>
       <c r="K92" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande; S4 Argument och kommunikation</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan; Formulera egna och granska andras argument; kommunicera</t>
         </is>
       </c>
       <c r="L92" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; SU3 Informationsgranskning; SU4 Argumentation</t>
+          <t>Hälsa; Informationsgranskning; Argumentation</t>
         </is>
       </c>
       <c r="M92" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -6204,17 +6204,17 @@
       </c>
       <c r="K93" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L93" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M93" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6267,17 +6267,17 @@
       </c>
       <c r="K94" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L94" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M94" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6330,17 +6330,17 @@
       </c>
       <c r="K95" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L95" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M95" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6393,17 +6393,17 @@
       </c>
       <c r="K96" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L96" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; KH3 Hälsa; SU1 Undersökningar</t>
+          <t>Celler och organsystem; Hälsa; Undersökningar</t>
         </is>
       </c>
       <c r="M96" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -6452,17 +6452,17 @@
       </c>
       <c r="K97" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L97" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Celler och organsystem; Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M97" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6511,17 +6511,17 @@
       </c>
       <c r="K98" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L98" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M98" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6570,17 +6570,17 @@
       </c>
       <c r="K99" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L99" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M99" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6629,17 +6629,17 @@
       </c>
       <c r="K100" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L100" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; KH3 Hälsa</t>
+          <t>Celler och organsystem; Hälsa</t>
         </is>
       </c>
       <c r="M100" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6692,17 +6692,17 @@
       </c>
       <c r="K101" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L101" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M101" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6755,17 +6755,17 @@
       </c>
       <c r="K102" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L102" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M102" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6818,17 +6818,17 @@
       </c>
       <c r="K103" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L103" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner; KH3 Hälsa</t>
+          <t>Infektioner; Hälsa</t>
         </is>
       </c>
       <c r="M103" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -6881,17 +6881,17 @@
       </c>
       <c r="K104" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner; SU1 Undersökningar</t>
+          <t>Infektioner; Undersökningar</t>
         </is>
       </c>
       <c r="M104" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -6940,17 +6940,17 @@
       </c>
       <c r="K105" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L105" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M105" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7003,17 +7003,17 @@
       </c>
       <c r="K106" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L106" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M106" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7066,17 +7066,17 @@
       </c>
       <c r="K107" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L107" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M107" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7129,17 +7129,17 @@
       </c>
       <c r="K108" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L108" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner; NM1 Evolution och mångfald</t>
+          <t>Infektioner; Evolution och mångfald</t>
         </is>
       </c>
       <c r="M108" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7192,17 +7192,17 @@
       </c>
       <c r="K109" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L109" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner; SU3 Informationsgranskning</t>
+          <t>Infektioner; Informationsgranskning</t>
         </is>
       </c>
       <c r="M109" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -7251,17 +7251,17 @@
       </c>
       <c r="K110" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L110" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M110" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7310,17 +7310,17 @@
       </c>
       <c r="K111" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L111" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M111" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7369,17 +7369,17 @@
       </c>
       <c r="K112" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L112" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner</t>
+          <t>Infektioner</t>
         </is>
       </c>
       <c r="M112" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7428,17 +7428,17 @@
       </c>
       <c r="K113" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande; S4 Argument och kommunikation</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan; Formulera egna och granska andras argument; kommunicera</t>
         </is>
       </c>
       <c r="L113" s="4" t="inlineStr">
         <is>
-          <t>KH2 Infektioner; SU3 Informationsgranskning; SU4 Argumentation</t>
+          <t>Infektioner; Informationsgranskning; Argumentation</t>
         </is>
       </c>
       <c r="M113" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -7491,17 +7491,17 @@
       </c>
       <c r="K114" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L114" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M114" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7554,17 +7554,17 @@
       </c>
       <c r="K115" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L115" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M115" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7617,17 +7617,17 @@
       </c>
       <c r="K116" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L116" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M116" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7680,17 +7680,17 @@
       </c>
       <c r="K117" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L117" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö; SU1 Undersökningar</t>
+          <t>Arv och miljö; Undersökningar</t>
         </is>
       </c>
       <c r="M117" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -7739,17 +7739,17 @@
       </c>
       <c r="K118" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L118" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M118" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7798,17 +7798,17 @@
       </c>
       <c r="K119" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L119" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M119" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7857,17 +7857,17 @@
       </c>
       <c r="K120" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L120" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö; KH1 Celler och organsystem</t>
+          <t>Arv och miljö; Celler och organsystem</t>
         </is>
       </c>
       <c r="M120" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7916,17 +7916,17 @@
       </c>
       <c r="K121" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L121" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M121" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -7975,17 +7975,17 @@
       </c>
       <c r="K122" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L122" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö; KH3 Hälsa</t>
+          <t>Arv och miljö; Hälsa</t>
         </is>
       </c>
       <c r="M122" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8038,17 +8038,17 @@
       </c>
       <c r="K123" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L123" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö</t>
+          <t>Arv och miljö</t>
         </is>
       </c>
       <c r="M123" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8101,17 +8101,17 @@
       </c>
       <c r="K124" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L124" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik</t>
+          <t>Genteknik</t>
         </is>
       </c>
       <c r="M124" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8164,17 +8164,17 @@
       </c>
       <c r="K125" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val; S4 Argument och kommunikation</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa; Formulera egna och granska andras argument; kommunicera</t>
         </is>
       </c>
       <c r="L125" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik; SU4 Argumentation</t>
+          <t>Genteknik; Argumentation</t>
         </is>
       </c>
       <c r="M125" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -8227,17 +8227,17 @@
       </c>
       <c r="K126" s="4" t="inlineStr">
         <is>
-          <t>S4 Argument och kommunikation; S5 Etiska val</t>
+          <t>Formulera egna och granska andras argument; kommunicera; Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L126" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik; SU4 Argumentation</t>
+          <t>Genteknik; Argumentation</t>
         </is>
       </c>
       <c r="M126" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -8286,17 +8286,17 @@
       </c>
       <c r="K127" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L127" s="4" t="inlineStr">
         <is>
-          <t>NM2 Arv och miljö; NM1 Evolution och mångfald</t>
+          <t>Arv och miljö; Evolution och mångfald</t>
         </is>
       </c>
       <c r="M127" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8345,17 +8345,17 @@
       </c>
       <c r="K128" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L128" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik</t>
+          <t>Genteknik</t>
         </is>
       </c>
       <c r="M128" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8404,17 +8404,17 @@
       </c>
       <c r="K129" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L129" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik</t>
+          <t>Genteknik</t>
         </is>
       </c>
       <c r="M129" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8463,17 +8463,17 @@
       </c>
       <c r="K130" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L130" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik</t>
+          <t>Genteknik</t>
         </is>
       </c>
       <c r="M130" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8522,17 +8522,17 @@
       </c>
       <c r="K131" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L131" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik</t>
+          <t>Genteknik</t>
         </is>
       </c>
       <c r="M131" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8581,17 +8581,17 @@
       </c>
       <c r="K132" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L132" s="4" t="inlineStr">
         <is>
-          <t>NM3 Genteknik</t>
+          <t>Genteknik</t>
         </is>
       </c>
       <c r="M132" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -8644,17 +8644,17 @@
       </c>
       <c r="K133" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L133" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M133" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8707,17 +8707,17 @@
       </c>
       <c r="K134" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L134" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M134" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8770,17 +8770,17 @@
       </c>
       <c r="K135" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L135" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; SU2 Modeller och historia</t>
+          <t>Evolution och mångfald; Modeller och historia</t>
         </is>
       </c>
       <c r="M135" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8833,17 +8833,17 @@
       </c>
       <c r="K136" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L136" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; SU2 Modeller och historia</t>
+          <t>Evolution och mångfald; Modeller och historia</t>
         </is>
       </c>
       <c r="M136" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -8892,17 +8892,17 @@
       </c>
       <c r="K137" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L137" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; SU2 Modeller och historia</t>
+          <t>Evolution och mångfald; Modeller och historia</t>
         </is>
       </c>
       <c r="M137" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -8951,17 +8951,17 @@
       </c>
       <c r="K138" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L138" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM2 Arv och miljö</t>
+          <t>Evolution och mångfald; Arv och miljö</t>
         </is>
       </c>
       <c r="M138" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9014,17 +9014,17 @@
       </c>
       <c r="K139" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L139" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM2 Arv och miljö</t>
+          <t>Evolution och mångfald; Arv och miljö</t>
         </is>
       </c>
       <c r="M139" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9077,17 +9077,17 @@
       </c>
       <c r="K140" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L140" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M140" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9140,13 +9140,13 @@
       </c>
       <c r="K141" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S6 Källor och kritiskt tänkande</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L141" s="4" t="inlineStr"/>
       <c r="M141" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -9199,17 +9199,17 @@
       </c>
       <c r="K142" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L142" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; SU1 Undersökningar; SU2 Modeller och historia</t>
+          <t>Evolution och mångfald; Undersökningar; Modeller och historia</t>
         </is>
       </c>
       <c r="M142" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -9258,17 +9258,17 @@
       </c>
       <c r="K143" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L143" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM2 Arv och miljö</t>
+          <t>Evolution och mångfald; Arv och miljö</t>
         </is>
       </c>
       <c r="M143" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9317,17 +9317,17 @@
       </c>
       <c r="K144" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L144" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald</t>
+          <t>Evolution och mångfald</t>
         </is>
       </c>
       <c r="M144" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9376,17 +9376,17 @@
       </c>
       <c r="K145" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L145" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; SU2 Modeller och historia</t>
+          <t>Evolution och mångfald; Modeller och historia</t>
         </is>
       </c>
       <c r="M145" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9439,17 +9439,17 @@
       </c>
       <c r="K146" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L146" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; KH1 Celler och organsystem</t>
+          <t>Hälsa; Celler och organsystem</t>
         </is>
       </c>
       <c r="M146" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9502,17 +9502,17 @@
       </c>
       <c r="K147" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L147" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M147" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9565,17 +9565,17 @@
       </c>
       <c r="K148" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L148" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M148" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9628,17 +9628,17 @@
       </c>
       <c r="K149" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar; S6 Källor och kritiskt tänkande</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder; Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L149" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; SU1 Undersökningar; SU3 Informationsgranskning</t>
+          <t>Hälsa; Undersökningar; Informationsgranskning</t>
         </is>
       </c>
       <c r="M149" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -9687,17 +9687,17 @@
       </c>
       <c r="K150" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L150" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M150" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9746,17 +9746,17 @@
       </c>
       <c r="K151" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L151" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem</t>
+          <t>Celler och organsystem</t>
         </is>
       </c>
       <c r="M151" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9806,12 +9806,12 @@
       <c r="K152" s="4" t="inlineStr"/>
       <c r="L152" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M152" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -9860,17 +9860,17 @@
       </c>
       <c r="K153" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L153" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M153" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9919,17 +9919,17 @@
       </c>
       <c r="K154" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L154" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M154" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -9982,17 +9982,17 @@
       </c>
       <c r="K155" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L155" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M155" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10045,17 +10045,17 @@
       </c>
       <c r="K156" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L156" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; KH1 Celler och organsystem</t>
+          <t>Hälsa; Celler och organsystem</t>
         </is>
       </c>
       <c r="M156" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10108,17 +10108,17 @@
       </c>
       <c r="K157" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val; S4 Argument och kommunikation</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa; Formulera egna och granska andras argument; kommunicera</t>
         </is>
       </c>
       <c r="L157" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; SU4 Argumentation</t>
+          <t>Hälsa; Argumentation</t>
         </is>
       </c>
       <c r="M157" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -10171,17 +10171,17 @@
       </c>
       <c r="K158" s="4" t="inlineStr">
         <is>
-          <t>S8 Material, utrustning, digitalt; S7 Systematiska undersökningar; S6 Källor och kritiskt tänkande</t>
+          <t>Färdigheter i att hantera material, utrustning och digitala verktyg; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder; Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L158" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa; SU1 Undersökningar; SU3 Informationsgranskning</t>
+          <t>Hälsa; Undersökningar; Informationsgranskning</t>
         </is>
       </c>
       <c r="M158" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -10230,17 +10230,17 @@
       </c>
       <c r="K159" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L159" s="4" t="inlineStr">
         <is>
-          <t>KH3 Hälsa</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="M159" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10293,17 +10293,17 @@
       </c>
       <c r="K160" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L160" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer; KH1 Celler och organsystem</t>
+          <t>Reproduktion och relationer; Celler och organsystem</t>
         </is>
       </c>
       <c r="M160" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10356,17 +10356,17 @@
       </c>
       <c r="K161" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L161" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M161" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10419,17 +10419,17 @@
       </c>
       <c r="K162" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L162" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer; KH2 Infektioner</t>
+          <t>Reproduktion och relationer; Infektioner</t>
         </is>
       </c>
       <c r="M162" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10482,17 +10482,17 @@
       </c>
       <c r="K163" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L163" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer; SU3 Informationsgranskning</t>
+          <t>Reproduktion och relationer; Informationsgranskning</t>
         </is>
       </c>
       <c r="M163" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -10541,17 +10541,17 @@
       </c>
       <c r="K164" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L164" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M164" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10600,17 +10600,17 @@
       </c>
       <c r="K165" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L165" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M165" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10659,17 +10659,17 @@
       </c>
       <c r="K166" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L166" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M166" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10718,17 +10718,17 @@
       </c>
       <c r="K167" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L167" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer; KH2 Infektioner</t>
+          <t>Reproduktion och relationer; Infektioner</t>
         </is>
       </c>
       <c r="M167" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10777,17 +10777,17 @@
       </c>
       <c r="K168" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L168" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M168" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10840,17 +10840,17 @@
       </c>
       <c r="K169" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L169" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M169" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -10903,17 +10903,17 @@
       </c>
       <c r="K170" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L170" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M170" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -10966,17 +10966,17 @@
       </c>
       <c r="K171" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L171" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer</t>
+          <t>Reproduktion och relationer</t>
         </is>
       </c>
       <c r="M171" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -11029,17 +11029,17 @@
       </c>
       <c r="K172" s="4" t="inlineStr">
         <is>
-          <t>S5 Etiska val; S4 Argument och kommunikation</t>
+          <t>Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa; Formulera egna och granska andras argument; kommunicera</t>
         </is>
       </c>
       <c r="L172" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer; SU4 Argumentation</t>
+          <t>Reproduktion och relationer; Argumentation</t>
         </is>
       </c>
       <c r="M172" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -11088,17 +11088,17 @@
       </c>
       <c r="K173" s="4" t="inlineStr">
         <is>
-          <t>S6 Källor och kritiskt tänkande</t>
+          <t>Söka svar med olika typer av källor; kritiskt tänkande och tilltro till den egna förmågan</t>
         </is>
       </c>
       <c r="L173" s="4" t="inlineStr">
         <is>
-          <t>KH4 Reproduktion och relationer; SU3 Informationsgranskning</t>
+          <t>Reproduktion och relationer; Informationsgranskning</t>
         </is>
       </c>
       <c r="M173" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -11151,17 +11151,17 @@
       </c>
       <c r="K174" s="4" t="inlineStr">
         <is>
-          <t>S3 Evolution och världsbild; S2 Begrepp och samband</t>
+          <t>Naturvetenskapens världsbild med evolutionsteorin som grund; skilja naturvetenskapliga från andra sätt att förklara omvärlden; Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L174" s="4" t="inlineStr">
         <is>
-          <t>NM1 Evolution och mångfald; NM5 Fotosyntes, kretslopp, energi</t>
+          <t>Evolution och mångfald; Fotosyntes, kretslopp, energi</t>
         </is>
       </c>
       <c r="M174" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -11214,17 +11214,17 @@
       </c>
       <c r="K175" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L175" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M175" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -11277,17 +11277,17 @@
       </c>
       <c r="K176" s="4" t="inlineStr">
         <is>
-          <t>S4 Argument och kommunikation; S5 Etiska val</t>
+          <t>Formulera egna och granska andras argument; kommunicera; Hantera praktiska och etiska valsituationer i frågor om miljö och hälsa</t>
         </is>
       </c>
       <c r="L176" s="4" t="inlineStr">
         <is>
-          <t>SU4 Argumentation</t>
+          <t>Argumentation</t>
         </is>
       </c>
       <c r="M176" s="4" t="inlineStr">
         <is>
-          <t>F2 Granska/ta ställning</t>
+          <t>Granska/ta ställning</t>
         </is>
       </c>
     </row>
@@ -11340,17 +11340,17 @@
       </c>
       <c r="K177" s="4" t="inlineStr">
         <is>
-          <t>S7 Systematiska undersökningar</t>
+          <t>Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L177" s="4" t="inlineStr">
         <is>
-          <t>SU1 Undersökningar</t>
+          <t>Undersökningar</t>
         </is>
       </c>
       <c r="M177" s="4" t="inlineStr">
         <is>
-          <t>F3 Undersöka</t>
+          <t>Undersöka</t>
         </is>
       </c>
     </row>
@@ -11399,17 +11399,17 @@
       </c>
       <c r="K178" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband</t>
         </is>
       </c>
       <c r="L178" s="4" t="inlineStr">
         <is>
-          <t>KH1 Celler och organsystem; KH2 Infektioner; KH3 Hälsa</t>
+          <t>Celler och organsystem; Infektioner; Hälsa</t>
         </is>
       </c>
       <c r="M178" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller</t>
+          <t>Begrepp/modeller</t>
         </is>
       </c>
     </row>
@@ -11458,13 +11458,13 @@
       </c>
       <c r="K179" s="4" t="inlineStr">
         <is>
-          <t>S2 Begrepp och samband; S7 Systematiska undersökningar</t>
+          <t>Kunskaper om natur och människokropp; använda begrepp och förklaringsmodeller för att beskriva och förklara samband; Egna systematiska undersökningar; påståenden kan prövas; kunskap växer fram med naturvetenskapliga arbetsmetoder</t>
         </is>
       </c>
       <c r="L179" s="4" t="inlineStr"/>
       <c r="M179" s="4" t="inlineStr">
         <is>
-          <t>F1 Begrepp/modeller; F2 Granska/ta ställning; F3 Undersöka</t>
+          <t>Begrepp/modeller; Granska/ta ställning; Undersöka</t>
         </is>
       </c>
     </row>

</xml_diff>